<commit_message>
atualização dos dados do 1Q26
</commit_message>
<xml_diff>
--- a/analise_eua/energia_eletrica/constellation/ceg_indicators.xlsx
+++ b/analise_eua/energia_eletrica/constellation/ceg_indicators.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,13 +49,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,166 +436,166 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>DPA</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Payout</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>2025</v>
       </c>
       <c r="B2" t="n">
-        <v>47.68</v>
+        <v>47.62</v>
       </c>
       <c r="C2" t="n">
-        <v>47.67</v>
+        <v>47.61</v>
       </c>
       <c r="D2" t="n">
         <v>2.1</v>
@@ -593,10 +607,10 @@
         <v>9.08</v>
       </c>
       <c r="G2" t="n">
-        <v>7.62</v>
+        <v>7.61</v>
       </c>
       <c r="H2" t="n">
-        <v>110573510</v>
+        <v>110426400</v>
       </c>
       <c r="I2" t="n">
         <v>8992</v>
@@ -614,7 +628,7 @@
         <v>0.36</v>
       </c>
       <c r="N2" t="n">
-        <v>20.37</v>
+        <v>20.34</v>
       </c>
       <c r="O2" t="n">
         <v>15.97</v>
@@ -669,17 +683,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>18.69</v>
+        <v>18.67</v>
       </c>
       <c r="C3" t="n">
-        <v>18.69</v>
+        <v>18.67</v>
       </c>
       <c r="D3" t="n">
-        <v>5.35</v>
+        <v>5.36</v>
       </c>
       <c r="E3" t="n">
         <v>7052</v>
@@ -691,7 +705,7 @@
         <v>5.32</v>
       </c>
       <c r="H3" t="n">
-        <v>70074900.00000001</v>
+        <v>69983550</v>
       </c>
       <c r="I3" t="n">
         <v>8412</v>
@@ -709,7 +723,7 @@
         <v>0.4</v>
       </c>
       <c r="N3" t="n">
-        <v>10.69</v>
+        <v>10.67</v>
       </c>
       <c r="O3" t="n">
         <v>28.47</v>
@@ -764,14 +778,14 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2023</v>
       </c>
       <c r="B4" t="n">
-        <v>22.97</v>
+        <v>22.94</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>22.96</v>
       </c>
       <c r="D4" t="n">
         <v>4.35</v>
@@ -786,7 +800,7 @@
         <v>3.41</v>
       </c>
       <c r="H4" t="n">
-        <v>37287120</v>
+        <v>37235440</v>
       </c>
       <c r="I4" t="n">
         <v>9261</v>
@@ -804,7 +818,7 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="N4" t="n">
-        <v>11.18</v>
+        <v>11.16</v>
       </c>
       <c r="O4" t="n">
         <v>14.86</v>
@@ -859,11 +873,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>-172.43</v>
+        <v>-172.2</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -881,7 +895,7 @@
         <v>2.5</v>
       </c>
       <c r="H5" t="n">
-        <v>27588080</v>
+        <v>27552000</v>
       </c>
       <c r="I5" t="n">
         <v>5768</v>
@@ -899,7 +913,7 @@
         <v>0.48</v>
       </c>
       <c r="N5" t="n">
-        <v>11.23</v>
+        <v>11.22</v>
       </c>
       <c r="O5" t="n">
         <v>-1.45</v>
@@ -964,1013 +978,1108 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>DPA</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Payout</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>45930</v>
+      <c r="A2" s="2" t="n">
+        <v>46112</v>
       </c>
       <c r="B2" t="n">
-        <v>110.62</v>
+        <v>62.17</v>
       </c>
       <c r="C2" t="n">
-        <v>33.37</v>
+        <v>26.57</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>3.76</v>
       </c>
       <c r="E2" t="n">
-        <v>1731</v>
+        <v>3534</v>
       </c>
       <c r="F2" t="n">
-        <v>14.16</v>
+        <v>14.3</v>
       </c>
       <c r="G2" t="n">
-        <v>7.17</v>
+        <v>2.95</v>
       </c>
       <c r="H2" t="n">
-        <v>102879970</v>
+        <v>98854500</v>
       </c>
       <c r="I2" t="n">
-        <v>7387</v>
+        <v>17364</v>
       </c>
       <c r="J2" t="n">
-        <v>4091</v>
+        <v>1171</v>
       </c>
       <c r="K2" t="n">
-        <v>3296</v>
+        <v>16193</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5</v>
+        <v>2.03</v>
       </c>
       <c r="M2" t="n">
-        <v>0.23</v>
+        <v>0.48</v>
       </c>
       <c r="N2" t="n">
-        <v>16.18</v>
+        <v>14.44</v>
       </c>
       <c r="O2" t="n">
-        <v>21.51</v>
+        <v>10.38</v>
       </c>
       <c r="P2" t="n">
-        <v>11.86</v>
+        <v>6.61</v>
       </c>
       <c r="Q2" t="n">
-        <v>1848</v>
+        <v>425</v>
       </c>
       <c r="R2" t="n">
-        <v>-463</v>
+        <v>-3732</v>
       </c>
       <c r="S2" t="n">
-        <v>644</v>
+        <v>730</v>
       </c>
       <c r="T2" t="n">
-        <v>1458</v>
+        <v>-850</v>
       </c>
       <c r="U2" t="n">
-        <v>390</v>
+        <v>1275</v>
       </c>
       <c r="V2" t="n">
-        <v>-91</v>
+        <v>91</v>
       </c>
       <c r="W2" t="n">
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>-91</v>
+        <v>91</v>
       </c>
       <c r="Y2" t="n">
-        <v>4194</v>
+        <v>4794</v>
       </c>
       <c r="Z2" t="n">
-        <v>-21.3</v>
+        <v>36.94</v>
       </c>
       <c r="AA2" t="n">
-        <v>4016</v>
+        <v>1865</v>
       </c>
       <c r="AB2" t="n">
-        <v>3183</v>
+        <v>2376</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.39</v>
+        <v>0.44</v>
       </c>
       <c r="AD2" t="n">
-        <v>13.12</v>
+        <v>9.75</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>45838</v>
+      <c r="A3" s="2" t="n">
+        <v>45930</v>
       </c>
       <c r="B3" t="n">
-        <v>120.51</v>
+        <v>110.48</v>
       </c>
       <c r="C3" t="n">
-        <v>34.04</v>
+        <v>33.32</v>
       </c>
       <c r="D3" t="n">
-        <v>2.94</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>1611</v>
+        <v>1731</v>
       </c>
       <c r="F3" t="n">
-        <v>13.75</v>
+        <v>14.16</v>
       </c>
       <c r="G3" t="n">
-        <v>7.52</v>
+        <v>7.16</v>
       </c>
       <c r="H3" t="n">
-        <v>101108000</v>
+        <v>102742250</v>
       </c>
       <c r="I3" t="n">
-        <v>7411</v>
+        <v>7387</v>
       </c>
       <c r="J3" t="n">
-        <v>2062</v>
+        <v>4091</v>
       </c>
       <c r="K3" t="n">
-        <v>5349</v>
+        <v>3296</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4</v>
+        <v>0.23</v>
       </c>
       <c r="N3" t="n">
-        <v>16.07</v>
+        <v>16.16</v>
       </c>
       <c r="O3" t="n">
-        <v>22.1</v>
+        <v>21.51</v>
       </c>
       <c r="P3" t="n">
-        <v>13.92</v>
+        <v>11.86</v>
       </c>
       <c r="Q3" t="n">
-        <v>1477</v>
+        <v>1848</v>
       </c>
       <c r="R3" t="n">
-        <v>-872</v>
+        <v>-463</v>
       </c>
       <c r="S3" t="n">
-        <v>-485</v>
+        <v>644</v>
       </c>
       <c r="T3" t="n">
-        <v>710</v>
+        <v>1458</v>
       </c>
       <c r="U3" t="n">
-        <v>767</v>
+        <v>390</v>
       </c>
       <c r="V3" t="n">
-        <v>16</v>
+        <v>-91</v>
       </c>
       <c r="W3" t="n">
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>16</v>
+        <v>-91</v>
       </c>
       <c r="Y3" t="n">
-        <v>2977</v>
+        <v>4194</v>
       </c>
       <c r="Z3" t="n">
-        <v>-16.84</v>
+        <v>-21.3</v>
       </c>
       <c r="AA3" t="n">
-        <v>3046</v>
+        <v>4016</v>
       </c>
       <c r="AB3" t="n">
-        <v>3086</v>
+        <v>3183</v>
       </c>
       <c r="AC3" t="n">
         <v>0.39</v>
       </c>
       <c r="AD3" t="n">
-        <v>14.54</v>
+        <v>13.12</v>
       </c>
       <c r="AE3" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>45747</v>
+      <c r="A4" s="2" t="n">
+        <v>45838</v>
       </c>
       <c r="B4" t="n">
-        <v>532.84</v>
+        <v>120.35</v>
       </c>
       <c r="C4" t="n">
-        <v>20.97</v>
+        <v>33.99</v>
       </c>
       <c r="D4" t="n">
-        <v>4.77</v>
+        <v>2.94</v>
       </c>
       <c r="E4" t="n">
-        <v>1091</v>
+        <v>1611</v>
       </c>
       <c r="F4" t="n">
-        <v>1.74</v>
+        <v>13.75</v>
       </c>
       <c r="G4" t="n">
-        <v>4.85</v>
+        <v>7.51</v>
       </c>
       <c r="H4" t="n">
-        <v>62875439.99999999</v>
+        <v>100972980</v>
       </c>
       <c r="I4" t="n">
-        <v>8358</v>
+        <v>7411</v>
       </c>
       <c r="J4" t="n">
-        <v>1942</v>
+        <v>2062</v>
       </c>
       <c r="K4" t="n">
-        <v>6416</v>
+        <v>5349</v>
       </c>
       <c r="L4" t="n">
-        <v>0.98</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="N4" t="n">
-        <v>10.63</v>
+        <v>16.05</v>
       </c>
       <c r="O4" t="n">
-        <v>23.27</v>
+        <v>22.1</v>
       </c>
       <c r="P4" t="n">
-        <v>14.27</v>
+        <v>13.92</v>
       </c>
       <c r="Q4" t="n">
-        <v>107</v>
+        <v>1477</v>
       </c>
       <c r="R4" t="n">
-        <v>-886</v>
+        <v>-872</v>
       </c>
       <c r="S4" t="n">
-        <v>-408</v>
+        <v>-485</v>
       </c>
       <c r="T4" t="n">
-        <v>-699</v>
+        <v>710</v>
       </c>
       <c r="U4" t="n">
-        <v>806</v>
+        <v>767</v>
       </c>
       <c r="V4" t="n">
-        <v>-47</v>
+        <v>16</v>
       </c>
       <c r="W4" t="n">
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>-47</v>
+        <v>16</v>
       </c>
       <c r="Y4" t="n">
+        <v>2977</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>-16.84</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>3046</v>
+      </c>
+      <c r="AB4" t="n">
         <v>3086</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>40.84</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>1978</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>2031</v>
       </c>
       <c r="AC4" t="n">
         <v>0.39</v>
       </c>
       <c r="AD4" t="n">
-        <v>103.39</v>
+        <v>14.54</v>
       </c>
       <c r="AE4" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>45565</v>
+      <c r="A5" s="2" t="n">
+        <v>45747</v>
       </c>
       <c r="B5" t="n">
-        <v>67.34</v>
+        <v>532.13</v>
       </c>
       <c r="C5" t="n">
-        <v>22.51</v>
+        <v>20.94</v>
       </c>
       <c r="D5" t="n">
-        <v>4.44</v>
+        <v>4.78</v>
       </c>
       <c r="E5" t="n">
-        <v>2128</v>
+        <v>1091</v>
       </c>
       <c r="F5" t="n">
-        <v>18.32</v>
+        <v>1.74</v>
       </c>
       <c r="G5" t="n">
-        <v>6.43</v>
+        <v>4.85</v>
       </c>
       <c r="H5" t="n">
-        <v>80807210</v>
+        <v>62790930.00000001</v>
       </c>
       <c r="I5" t="n">
-        <v>8412</v>
+        <v>8358</v>
       </c>
       <c r="J5" t="n">
-        <v>1882</v>
+        <v>1942</v>
       </c>
       <c r="K5" t="n">
-        <v>6530</v>
+        <v>6416</v>
       </c>
       <c r="L5" t="n">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
       <c r="M5" t="n">
-        <v>0.52</v>
+        <v>0.5</v>
       </c>
       <c r="N5" t="n">
-        <v>12.43</v>
+        <v>10.61</v>
       </c>
       <c r="O5" t="n">
-        <v>28.86</v>
+        <v>23.27</v>
       </c>
       <c r="P5" t="n">
-        <v>16.13</v>
+        <v>14.27</v>
       </c>
       <c r="Q5" t="n">
-        <v>-112</v>
+        <v>107</v>
       </c>
       <c r="R5" t="n">
-        <v>2406</v>
+        <v>-886</v>
       </c>
       <c r="S5" t="n">
-        <v>-795</v>
+        <v>-408</v>
       </c>
       <c r="T5" t="n">
-        <v>-664</v>
+        <v>-699</v>
       </c>
       <c r="U5" t="n">
-        <v>552</v>
+        <v>806</v>
       </c>
       <c r="V5" t="n">
-        <v>-435</v>
+        <v>-47</v>
       </c>
       <c r="W5" t="n">
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>-435</v>
+        <v>-47</v>
       </c>
       <c r="Y5" t="n">
-        <v>3818</v>
+        <v>3086</v>
       </c>
       <c r="Z5" t="n">
-        <v>25.98</v>
+        <v>40.84</v>
       </c>
       <c r="AA5" t="n">
-        <v>4410</v>
+        <v>1978</v>
       </c>
       <c r="AB5" t="n">
-        <v>2289</v>
+        <v>2031</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.35</v>
+        <v>0.39</v>
       </c>
       <c r="AD5" t="n">
-        <v>9.25</v>
+        <v>103.39</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>45473</v>
+      <c r="A6" s="2" t="n">
+        <v>45565</v>
       </c>
       <c r="B6" t="n">
-        <v>76.8</v>
+        <v>67.25</v>
       </c>
       <c r="C6" t="n">
-        <v>19.44</v>
+        <v>22.48</v>
       </c>
       <c r="D6" t="n">
-        <v>5.14</v>
+        <v>4.45</v>
       </c>
       <c r="E6" t="n">
-        <v>1794</v>
+        <v>2128</v>
       </c>
       <c r="F6" t="n">
-        <v>14.87</v>
+        <v>18.32</v>
       </c>
       <c r="G6" t="n">
-        <v>5.47</v>
+        <v>6.42</v>
       </c>
       <c r="H6" t="n">
-        <v>62518050</v>
+        <v>80697660</v>
       </c>
       <c r="I6" t="n">
-        <v>8444</v>
+        <v>8412</v>
       </c>
       <c r="J6" t="n">
-        <v>383</v>
+        <v>1882</v>
       </c>
       <c r="K6" t="n">
-        <v>8061</v>
+        <v>6530</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3</v>
+        <v>0.93</v>
       </c>
       <c r="M6" t="n">
-        <v>0.71</v>
+        <v>0.52</v>
       </c>
       <c r="N6" t="n">
-        <v>11.42</v>
+        <v>12.41</v>
       </c>
       <c r="O6" t="n">
-        <v>28.54</v>
+        <v>28.86</v>
       </c>
       <c r="P6" t="n">
-        <v>13.55</v>
+        <v>16.13</v>
       </c>
       <c r="Q6" t="n">
-        <v>-613</v>
+        <v>-112</v>
       </c>
       <c r="R6" t="n">
-        <v>1820</v>
+        <v>2406</v>
       </c>
       <c r="S6" t="n">
-        <v>-1469</v>
+        <v>-795</v>
       </c>
       <c r="T6" t="n">
-        <v>-1159</v>
+        <v>-664</v>
       </c>
       <c r="U6" t="n">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="V6" t="n">
-        <v>-264</v>
+        <v>-435</v>
       </c>
       <c r="W6" t="n">
         <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>-264</v>
+        <v>-435</v>
       </c>
       <c r="Y6" t="n">
-        <v>2051</v>
+        <v>3818</v>
       </c>
       <c r="Z6" t="n">
-        <v>47.94</v>
+        <v>25.98</v>
       </c>
       <c r="AA6" t="n">
-        <v>4212</v>
+        <v>4410</v>
       </c>
       <c r="AB6" t="n">
-        <v>1699</v>
+        <v>2289</v>
       </c>
       <c r="AC6" t="n">
         <v>0.35</v>
       </c>
       <c r="AD6" t="n">
-        <v>13.51</v>
+        <v>9.25</v>
       </c>
       <c r="AE6" t="n">
-        <v>500000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>45382</v>
+      <c r="A7" s="2" t="n">
+        <v>45473</v>
       </c>
       <c r="B7" t="n">
-        <v>65.67</v>
+        <v>76.7</v>
       </c>
       <c r="C7" t="n">
-        <v>23.09</v>
+        <v>19.41</v>
       </c>
       <c r="D7" t="n">
-        <v>4.33</v>
+        <v>5.15</v>
       </c>
       <c r="E7" t="n">
-        <v>1507</v>
+        <v>1794</v>
       </c>
       <c r="F7" t="n">
-        <v>14.33</v>
+        <v>14.87</v>
       </c>
       <c r="G7" t="n">
-        <v>5.18</v>
+        <v>5.46</v>
       </c>
       <c r="H7" t="n">
-        <v>57982470</v>
+        <v>62436150</v>
       </c>
       <c r="I7" t="n">
-        <v>8474</v>
+        <v>8444</v>
       </c>
       <c r="J7" t="n">
-        <v>645</v>
+        <v>383</v>
       </c>
       <c r="K7" t="n">
-        <v>7829</v>
+        <v>8061</v>
       </c>
       <c r="L7" t="n">
-        <v>1.56</v>
+        <v>1.3</v>
       </c>
       <c r="M7" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="N7" t="n">
-        <v>13.1</v>
+        <v>11.4</v>
       </c>
       <c r="O7" t="n">
-        <v>22.71</v>
+        <v>28.54</v>
       </c>
       <c r="P7" t="n">
-        <v>8.369999999999999</v>
+        <v>13.55</v>
       </c>
       <c r="Q7" t="n">
-        <v>-723</v>
+        <v>-613</v>
       </c>
       <c r="R7" t="n">
-        <v>830</v>
+        <v>1820</v>
       </c>
       <c r="S7" t="n">
-        <v>84</v>
+        <v>-1469</v>
       </c>
       <c r="T7" t="n">
-        <v>-1461</v>
+        <v>-1159</v>
       </c>
       <c r="U7" t="n">
-        <v>738</v>
+        <v>546</v>
       </c>
       <c r="V7" t="n">
-        <v>-61</v>
+        <v>-264</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>-61</v>
+        <v>-264</v>
       </c>
       <c r="Y7" t="n">
-        <v>2538</v>
+        <v>2051</v>
       </c>
       <c r="Z7" t="n">
-        <v>107.65</v>
+        <v>47.94</v>
       </c>
       <c r="AA7" t="n">
-        <v>4707</v>
+        <v>4212</v>
       </c>
       <c r="AB7" t="n">
-        <v>325</v>
+        <v>1699</v>
       </c>
       <c r="AC7" t="n">
         <v>0.35</v>
       </c>
       <c r="AD7" t="n">
-        <v>12.68</v>
+        <v>13.51</v>
       </c>
       <c r="AE7" t="n">
-        <v>499000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>45199</v>
+      <c r="A8" s="2" t="n">
+        <v>45382</v>
       </c>
       <c r="B8" t="n">
-        <v>47.34</v>
+        <v>65.58</v>
       </c>
       <c r="C8" t="n">
-        <v>23.57</v>
+        <v>23.06</v>
       </c>
       <c r="D8" t="n">
-        <v>4.24</v>
+        <v>4.34</v>
       </c>
       <c r="E8" t="n">
-        <v>1598</v>
+        <v>1507</v>
       </c>
       <c r="F8" t="n">
-        <v>11.96</v>
+        <v>14.33</v>
       </c>
       <c r="G8" t="n">
-        <v>2.97</v>
+        <v>5.17</v>
       </c>
       <c r="H8" t="n">
-        <v>34608560</v>
+        <v>57906390</v>
       </c>
       <c r="I8" t="n">
-        <v>7628</v>
+        <v>8474</v>
       </c>
       <c r="J8" t="n">
-        <v>1977</v>
+        <v>645</v>
       </c>
       <c r="K8" t="n">
-        <v>5651</v>
+        <v>7829</v>
       </c>
       <c r="L8" t="n">
-        <v>1.39</v>
+        <v>1.56</v>
       </c>
       <c r="M8" t="n">
-        <v>0.48</v>
+        <v>0.7</v>
       </c>
       <c r="N8" t="n">
-        <v>9.869999999999999</v>
+        <v>13.08</v>
       </c>
       <c r="O8" t="n">
-        <v>12.62</v>
+        <v>22.71</v>
       </c>
       <c r="P8" t="n">
-        <v>5.6</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>-993</v>
+        <v>-723</v>
       </c>
       <c r="R8" t="n">
-        <v>2008</v>
+        <v>830</v>
       </c>
       <c r="S8" t="n">
-        <v>637</v>
+        <v>84</v>
       </c>
       <c r="T8" t="n">
-        <v>-1392</v>
+        <v>-1461</v>
       </c>
       <c r="U8" t="n">
-        <v>399</v>
+        <v>738</v>
       </c>
       <c r="V8" t="n">
-        <v>-418</v>
+        <v>-61</v>
       </c>
       <c r="W8" t="n">
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>-418</v>
+        <v>-61</v>
       </c>
       <c r="Y8" t="n">
-        <v>4639</v>
+        <v>2538</v>
       </c>
       <c r="Z8" t="n">
-        <v>172.16</v>
+        <v>107.65</v>
       </c>
       <c r="AA8" t="n">
-        <v>2949</v>
+        <v>4707</v>
       </c>
       <c r="AB8" t="n">
-        <v>-600</v>
+        <v>325</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.29</v>
+        <v>0.35</v>
       </c>
       <c r="AD8" t="n">
-        <v>12.59</v>
+        <v>12.68</v>
       </c>
       <c r="AE8" t="n">
-        <v>251000</v>
+        <v>499000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>45107</v>
+      <c r="A9" s="2" t="n">
+        <v>45199</v>
       </c>
       <c r="B9" t="n">
-        <v>34.99</v>
+        <v>47.28</v>
       </c>
       <c r="C9" t="n">
-        <v>46.13</v>
+        <v>23.54</v>
       </c>
       <c r="D9" t="n">
-        <v>2.17</v>
+        <v>4.25</v>
       </c>
       <c r="E9" t="n">
-        <v>1283</v>
+        <v>1598</v>
       </c>
       <c r="F9" t="n">
-        <v>15.3</v>
+        <v>11.96</v>
       </c>
       <c r="G9" t="n">
-        <v>2.59</v>
+        <v>2.96</v>
       </c>
       <c r="H9" t="n">
-        <v>29147040</v>
+        <v>34560260</v>
       </c>
       <c r="I9" t="n">
-        <v>6266</v>
+        <v>7628</v>
       </c>
       <c r="J9" t="n">
-        <v>325</v>
+        <v>1977</v>
       </c>
       <c r="K9" t="n">
-        <v>5941</v>
+        <v>5651</v>
       </c>
       <c r="L9" t="n">
-        <v>1.77</v>
+        <v>1.39</v>
       </c>
       <c r="M9" t="n">
-        <v>0.53</v>
+        <v>0.48</v>
       </c>
       <c r="N9" t="n">
-        <v>10.45</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="O9" t="n">
+        <v>12.62</v>
+      </c>
+      <c r="P9" t="n">
         <v>5.6</v>
       </c>
-      <c r="P9" t="n">
-        <v>5.19</v>
-      </c>
       <c r="Q9" t="n">
-        <v>-192</v>
+        <v>-993</v>
       </c>
       <c r="R9" t="n">
-        <v>-48</v>
+        <v>2008</v>
       </c>
       <c r="S9" t="n">
-        <v>229</v>
+        <v>637</v>
       </c>
       <c r="T9" t="n">
-        <v>-868</v>
+        <v>-1392</v>
       </c>
       <c r="U9" t="n">
-        <v>676</v>
+        <v>399</v>
       </c>
       <c r="V9" t="n">
-        <v>-411</v>
+        <v>-418</v>
       </c>
       <c r="W9" t="n">
         <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>-411</v>
+        <v>-418</v>
       </c>
       <c r="Y9" t="n">
-        <v>2350</v>
+        <v>4639</v>
       </c>
       <c r="Z9" t="n">
-        <v>85.15000000000001</v>
+        <v>172.16</v>
       </c>
       <c r="AA9" t="n">
-        <v>868</v>
+        <v>2949</v>
       </c>
       <c r="AB9" t="n">
-        <v>-115</v>
+        <v>-600</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.28</v>
+        <v>0.29</v>
       </c>
       <c r="AD9" t="n">
-        <v>11.04</v>
+        <v>12.59</v>
       </c>
       <c r="AE9" t="n">
-        <v>268000</v>
+        <v>251000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>45016</v>
+      <c r="A10" s="2" t="n">
+        <v>45107</v>
       </c>
       <c r="B10" t="n">
-        <v>262.64</v>
+        <v>34.94</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>46.07</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.39</v>
+        <v>2.17</v>
       </c>
       <c r="E10" t="n">
-        <v>636</v>
+        <v>1283</v>
       </c>
       <c r="F10" t="n">
-        <v>1.27</v>
+        <v>15.3</v>
       </c>
       <c r="G10" t="n">
-        <v>2.35</v>
+        <v>2.59</v>
       </c>
       <c r="H10" t="n">
-        <v>25213360</v>
+        <v>29108160</v>
       </c>
       <c r="I10" t="n">
-        <v>5924</v>
+        <v>6266</v>
       </c>
       <c r="J10" t="n">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="K10" t="n">
-        <v>5588</v>
+        <v>5941</v>
       </c>
       <c r="L10" t="n">
-        <v>1.8</v>
+        <v>1.77</v>
       </c>
       <c r="M10" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="N10" t="n">
-        <v>9.9</v>
+        <v>10.44</v>
       </c>
       <c r="O10" t="n">
-        <v>-0.9</v>
+        <v>5.6</v>
       </c>
       <c r="P10" t="n">
-        <v>6.43</v>
+        <v>5.19</v>
       </c>
       <c r="Q10" t="n">
-        <v>-934</v>
+        <v>-192</v>
       </c>
       <c r="R10" t="n">
-        <v>219</v>
+        <v>-48</v>
       </c>
       <c r="S10" t="n">
-        <v>523</v>
+        <v>229</v>
       </c>
       <c r="T10" t="n">
-        <v>-1594</v>
+        <v>-868</v>
       </c>
       <c r="U10" t="n">
-        <v>660</v>
+        <v>676</v>
       </c>
       <c r="V10" t="n">
-        <v>-665</v>
+        <v>-411</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>-665</v>
+        <v>-411</v>
       </c>
       <c r="Y10" t="n">
-        <v>2161</v>
+        <v>2350</v>
       </c>
       <c r="Z10" t="n">
-        <v>102.34</v>
+        <v>85.15000000000001</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1883</v>
+        <v>868</v>
       </c>
       <c r="AB10" t="n">
-        <v>-782</v>
+        <v>-115</v>
       </c>
       <c r="AC10" t="n">
         <v>0.28</v>
       </c>
       <c r="AD10" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>268000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>45016</v>
+      </c>
+      <c r="B11" t="n">
+        <v>262.26</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="E11" t="n">
+        <v>636</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="H11" t="n">
+        <v>25177280</v>
+      </c>
+      <c r="I11" t="n">
+        <v>5924</v>
+      </c>
+      <c r="J11" t="n">
+        <v>336</v>
+      </c>
+      <c r="K11" t="n">
+        <v>5588</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="N11" t="n">
+        <v>9.890000000000001</v>
+      </c>
+      <c r="O11" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="P11" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>-934</v>
+      </c>
+      <c r="R11" t="n">
+        <v>219</v>
+      </c>
+      <c r="S11" t="n">
+        <v>523</v>
+      </c>
+      <c r="T11" t="n">
+        <v>-1594</v>
+      </c>
+      <c r="U11" t="n">
+        <v>660</v>
+      </c>
+      <c r="V11" t="n">
+        <v>-665</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
+        <v>-665</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>2161</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>102.34</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>-1883</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>-782</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="AD11" t="n">
         <v>96.88</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AE11" t="n">
         <v>231000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
atualizei os dados do 2Q26 da CEG
</commit_message>
<xml_diff>
--- a/analise_eua/energia_eletrica/constellation/ceg_indicators.xlsx
+++ b/analise_eua/energia_eletrica/constellation/ceg_indicators.xlsx
@@ -592,10 +592,10 @@
         <v>2025</v>
       </c>
       <c r="B2" t="n">
-        <v>47.62</v>
+        <v>47.54</v>
       </c>
       <c r="C2" t="n">
-        <v>47.61</v>
+        <v>47.54</v>
       </c>
       <c r="D2" t="n">
         <v>2.1</v>
@@ -607,10 +607,10 @@
         <v>9.08</v>
       </c>
       <c r="G2" t="n">
-        <v>7.61</v>
+        <v>7.59</v>
       </c>
       <c r="H2" t="n">
-        <v>110426400</v>
+        <v>110254250</v>
       </c>
       <c r="I2" t="n">
         <v>8992</v>
@@ -628,7 +628,7 @@
         <v>0.36</v>
       </c>
       <c r="N2" t="n">
-        <v>20.34</v>
+        <v>20.31</v>
       </c>
       <c r="O2" t="n">
         <v>15.97</v>
@@ -687,10 +687,10 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>18.67</v>
+        <v>18.64</v>
       </c>
       <c r="C3" t="n">
-        <v>18.67</v>
+        <v>18.64</v>
       </c>
       <c r="D3" t="n">
         <v>5.36</v>
@@ -702,10 +702,10 @@
         <v>15.91</v>
       </c>
       <c r="G3" t="n">
-        <v>5.32</v>
+        <v>5.31</v>
       </c>
       <c r="H3" t="n">
-        <v>69983550</v>
+        <v>69873300</v>
       </c>
       <c r="I3" t="n">
         <v>8412</v>
@@ -723,7 +723,7 @@
         <v>0.4</v>
       </c>
       <c r="N3" t="n">
-        <v>10.67</v>
+        <v>10.66</v>
       </c>
       <c r="O3" t="n">
         <v>28.47</v>
@@ -782,13 +782,13 @@
         <v>2023</v>
       </c>
       <c r="B4" t="n">
-        <v>22.94</v>
+        <v>22.91</v>
       </c>
       <c r="C4" t="n">
-        <v>22.96</v>
+        <v>22.93</v>
       </c>
       <c r="D4" t="n">
-        <v>4.35</v>
+        <v>4.36</v>
       </c>
       <c r="E4" t="n">
         <v>4124</v>
@@ -797,10 +797,10 @@
         <v>6.51</v>
       </c>
       <c r="G4" t="n">
-        <v>3.41</v>
+        <v>3.4</v>
       </c>
       <c r="H4" t="n">
-        <v>37235440</v>
+        <v>37177299.99999999</v>
       </c>
       <c r="I4" t="n">
         <v>9261</v>
@@ -818,7 +818,7 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="N4" t="n">
-        <v>11.16</v>
+        <v>11.15</v>
       </c>
       <c r="O4" t="n">
         <v>14.86</v>
@@ -877,7 +877,7 @@
         <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>-172.2</v>
+        <v>-171.93</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -895,7 +895,7 @@
         <v>2.5</v>
       </c>
       <c r="H5" t="n">
-        <v>27552000</v>
+        <v>27509360</v>
       </c>
       <c r="I5" t="n">
         <v>5768</v>
@@ -913,7 +913,7 @@
         <v>0.48</v>
       </c>
       <c r="N5" t="n">
-        <v>11.22</v>
+        <v>11.21</v>
       </c>
       <c r="O5" t="n">
         <v>-1.45</v>
@@ -978,7 +978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1135,189 +1135,189 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46112</v>
+        <v>46203</v>
       </c>
       <c r="B2" t="n">
-        <v>62.17</v>
+        <v>174.29</v>
       </c>
       <c r="C2" t="n">
-        <v>26.57</v>
+        <v>21.5</v>
       </c>
       <c r="D2" t="n">
-        <v>3.76</v>
+        <v>4.65</v>
       </c>
       <c r="E2" t="n">
-        <v>3534</v>
+        <v>1746</v>
       </c>
       <c r="F2" t="n">
-        <v>14.3</v>
+        <v>6.84</v>
       </c>
       <c r="G2" t="n">
-        <v>2.95</v>
+        <v>2.8</v>
       </c>
       <c r="H2" t="n">
-        <v>98854500</v>
+        <v>89413200</v>
       </c>
       <c r="I2" t="n">
-        <v>17364</v>
+        <v>19474</v>
       </c>
       <c r="J2" t="n">
-        <v>1171</v>
+        <v>1077</v>
       </c>
       <c r="K2" t="n">
-        <v>16193</v>
+        <v>18397</v>
       </c>
       <c r="L2" t="n">
-        <v>2.03</v>
+        <v>2.13</v>
       </c>
       <c r="M2" t="n">
-        <v>0.48</v>
+        <v>0.58</v>
       </c>
       <c r="N2" t="n">
-        <v>14.44</v>
+        <v>12.5</v>
       </c>
       <c r="O2" t="n">
-        <v>10.38</v>
+        <v>12.11</v>
       </c>
       <c r="P2" t="n">
-        <v>6.61</v>
+        <v>6.05</v>
       </c>
       <c r="Q2" t="n">
-        <v>425</v>
+        <v>1128</v>
       </c>
       <c r="R2" t="n">
-        <v>-3732</v>
+        <v>-1369</v>
       </c>
       <c r="S2" t="n">
-        <v>730</v>
+        <v>147</v>
       </c>
       <c r="T2" t="n">
-        <v>-850</v>
+        <v>-118</v>
       </c>
       <c r="U2" t="n">
-        <v>1275</v>
+        <v>1246</v>
       </c>
       <c r="V2" t="n">
-        <v>91</v>
+        <v>5</v>
       </c>
       <c r="W2" t="n">
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>91</v>
+        <v>5</v>
       </c>
       <c r="Y2" t="n">
-        <v>4794</v>
+        <v>5933</v>
       </c>
       <c r="Z2" t="n">
-        <v>36.94</v>
+        <v>17.85</v>
       </c>
       <c r="AA2" t="n">
-        <v>1865</v>
+        <v>4636</v>
       </c>
       <c r="AB2" t="n">
-        <v>2376</v>
+        <v>2204</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="AD2" t="n">
-        <v>9.75</v>
+        <v>30.02</v>
       </c>
       <c r="AE2" t="n">
-        <v>0</v>
+        <v>1971</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45930</v>
+        <v>46112</v>
       </c>
       <c r="B3" t="n">
-        <v>110.48</v>
+        <v>62.08</v>
       </c>
       <c r="C3" t="n">
-        <v>33.32</v>
+        <v>26.53</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>3.77</v>
       </c>
       <c r="E3" t="n">
-        <v>1731</v>
+        <v>3534</v>
       </c>
       <c r="F3" t="n">
-        <v>14.16</v>
+        <v>14.3</v>
       </c>
       <c r="G3" t="n">
-        <v>7.16</v>
+        <v>2.95</v>
       </c>
       <c r="H3" t="n">
-        <v>102742250</v>
+        <v>98702280</v>
       </c>
       <c r="I3" t="n">
-        <v>7387</v>
+        <v>17364</v>
       </c>
       <c r="J3" t="n">
-        <v>4091</v>
+        <v>1171</v>
       </c>
       <c r="K3" t="n">
-        <v>3296</v>
+        <v>16193</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5</v>
+        <v>2.03</v>
       </c>
       <c r="M3" t="n">
-        <v>0.23</v>
+        <v>0.48</v>
       </c>
       <c r="N3" t="n">
-        <v>16.16</v>
+        <v>14.42</v>
       </c>
       <c r="O3" t="n">
-        <v>21.51</v>
+        <v>10.38</v>
       </c>
       <c r="P3" t="n">
-        <v>11.86</v>
+        <v>6.61</v>
       </c>
       <c r="Q3" t="n">
-        <v>1848</v>
+        <v>425</v>
       </c>
       <c r="R3" t="n">
-        <v>-463</v>
+        <v>-3732</v>
       </c>
       <c r="S3" t="n">
-        <v>644</v>
+        <v>730</v>
       </c>
       <c r="T3" t="n">
-        <v>1458</v>
+        <v>-850</v>
       </c>
       <c r="U3" t="n">
-        <v>390</v>
+        <v>1275</v>
       </c>
       <c r="V3" t="n">
-        <v>-91</v>
+        <v>91</v>
       </c>
       <c r="W3" t="n">
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>-91</v>
+        <v>91</v>
       </c>
       <c r="Y3" t="n">
-        <v>4194</v>
+        <v>4794</v>
       </c>
       <c r="Z3" t="n">
-        <v>-21.3</v>
+        <v>36.94</v>
       </c>
       <c r="AA3" t="n">
-        <v>4016</v>
+        <v>1865</v>
       </c>
       <c r="AB3" t="n">
-        <v>3183</v>
+        <v>2376</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.39</v>
+        <v>0.44</v>
       </c>
       <c r="AD3" t="n">
-        <v>13.12</v>
+        <v>9.75</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
@@ -1325,284 +1325,284 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45838</v>
+        <v>45930</v>
       </c>
       <c r="B4" t="n">
-        <v>120.35</v>
+        <v>110.3</v>
       </c>
       <c r="C4" t="n">
-        <v>33.99</v>
+        <v>33.27</v>
       </c>
       <c r="D4" t="n">
-        <v>2.94</v>
+        <v>3.01</v>
       </c>
       <c r="E4" t="n">
-        <v>1611</v>
+        <v>1731</v>
       </c>
       <c r="F4" t="n">
-        <v>13.75</v>
+        <v>14.16</v>
       </c>
       <c r="G4" t="n">
-        <v>7.51</v>
+        <v>7.15</v>
       </c>
       <c r="H4" t="n">
-        <v>100972980</v>
+        <v>102582620</v>
       </c>
       <c r="I4" t="n">
-        <v>7411</v>
+        <v>7387</v>
       </c>
       <c r="J4" t="n">
-        <v>2062</v>
+        <v>4091</v>
       </c>
       <c r="K4" t="n">
-        <v>5349</v>
+        <v>3296</v>
       </c>
       <c r="L4" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="M4" t="n">
-        <v>0.4</v>
+        <v>0.23</v>
       </c>
       <c r="N4" t="n">
-        <v>16.05</v>
+        <v>16.14</v>
       </c>
       <c r="O4" t="n">
-        <v>22.1</v>
+        <v>21.51</v>
       </c>
       <c r="P4" t="n">
-        <v>13.92</v>
+        <v>11.86</v>
       </c>
       <c r="Q4" t="n">
-        <v>1477</v>
+        <v>1848</v>
       </c>
       <c r="R4" t="n">
-        <v>-872</v>
+        <v>-463</v>
       </c>
       <c r="S4" t="n">
-        <v>-485</v>
+        <v>644</v>
       </c>
       <c r="T4" t="n">
-        <v>710</v>
+        <v>1458</v>
       </c>
       <c r="U4" t="n">
-        <v>767</v>
+        <v>390</v>
       </c>
       <c r="V4" t="n">
-        <v>16</v>
+        <v>-91</v>
       </c>
       <c r="W4" t="n">
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>16</v>
+        <v>-91</v>
       </c>
       <c r="Y4" t="n">
-        <v>2977</v>
+        <v>4194</v>
       </c>
       <c r="Z4" t="n">
-        <v>-16.84</v>
+        <v>-21.3</v>
       </c>
       <c r="AA4" t="n">
-        <v>3046</v>
+        <v>4016</v>
       </c>
       <c r="AB4" t="n">
-        <v>3086</v>
+        <v>3183</v>
       </c>
       <c r="AC4" t="n">
         <v>0.39</v>
       </c>
       <c r="AD4" t="n">
-        <v>14.54</v>
+        <v>13.12</v>
       </c>
       <c r="AE4" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45747</v>
+        <v>45838</v>
       </c>
       <c r="B5" t="n">
-        <v>532.13</v>
+        <v>120.16</v>
       </c>
       <c r="C5" t="n">
-        <v>20.94</v>
+        <v>33.94</v>
       </c>
       <c r="D5" t="n">
-        <v>4.78</v>
+        <v>2.95</v>
       </c>
       <c r="E5" t="n">
-        <v>1091</v>
+        <v>1611</v>
       </c>
       <c r="F5" t="n">
-        <v>1.74</v>
+        <v>13.75</v>
       </c>
       <c r="G5" t="n">
-        <v>4.85</v>
+        <v>7.5</v>
       </c>
       <c r="H5" t="n">
-        <v>62790930.00000001</v>
+        <v>100815980</v>
       </c>
       <c r="I5" t="n">
-        <v>8358</v>
+        <v>7411</v>
       </c>
       <c r="J5" t="n">
-        <v>1942</v>
+        <v>2062</v>
       </c>
       <c r="K5" t="n">
-        <v>6416</v>
+        <v>5349</v>
       </c>
       <c r="L5" t="n">
-        <v>0.98</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="N5" t="n">
-        <v>10.61</v>
+        <v>16.03</v>
       </c>
       <c r="O5" t="n">
-        <v>23.27</v>
+        <v>22.1</v>
       </c>
       <c r="P5" t="n">
-        <v>14.27</v>
+        <v>13.92</v>
       </c>
       <c r="Q5" t="n">
-        <v>107</v>
+        <v>1477</v>
       </c>
       <c r="R5" t="n">
-        <v>-886</v>
+        <v>-872</v>
       </c>
       <c r="S5" t="n">
-        <v>-408</v>
+        <v>-485</v>
       </c>
       <c r="T5" t="n">
-        <v>-699</v>
+        <v>710</v>
       </c>
       <c r="U5" t="n">
-        <v>806</v>
+        <v>767</v>
       </c>
       <c r="V5" t="n">
-        <v>-47</v>
+        <v>16</v>
       </c>
       <c r="W5" t="n">
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>-47</v>
+        <v>16</v>
       </c>
       <c r="Y5" t="n">
+        <v>2977</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>-16.84</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>3046</v>
+      </c>
+      <c r="AB5" t="n">
         <v>3086</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>40.84</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>1978</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>2031</v>
       </c>
       <c r="AC5" t="n">
         <v>0.39</v>
       </c>
       <c r="AD5" t="n">
-        <v>103.39</v>
+        <v>14.54</v>
       </c>
       <c r="AE5" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45565</v>
+        <v>45747</v>
       </c>
       <c r="B6" t="n">
-        <v>67.25</v>
+        <v>531.3</v>
       </c>
       <c r="C6" t="n">
-        <v>22.48</v>
+        <v>20.91</v>
       </c>
       <c r="D6" t="n">
-        <v>4.45</v>
+        <v>4.78</v>
       </c>
       <c r="E6" t="n">
-        <v>2128</v>
+        <v>1091</v>
       </c>
       <c r="F6" t="n">
-        <v>18.32</v>
+        <v>1.74</v>
       </c>
       <c r="G6" t="n">
-        <v>6.42</v>
+        <v>4.84</v>
       </c>
       <c r="H6" t="n">
-        <v>80697660</v>
+        <v>62693900</v>
       </c>
       <c r="I6" t="n">
-        <v>8412</v>
+        <v>8358</v>
       </c>
       <c r="J6" t="n">
-        <v>1882</v>
+        <v>1942</v>
       </c>
       <c r="K6" t="n">
-        <v>6530</v>
+        <v>6416</v>
       </c>
       <c r="L6" t="n">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
       <c r="M6" t="n">
-        <v>0.52</v>
+        <v>0.5</v>
       </c>
       <c r="N6" t="n">
-        <v>12.41</v>
+        <v>10.6</v>
       </c>
       <c r="O6" t="n">
-        <v>28.86</v>
+        <v>23.27</v>
       </c>
       <c r="P6" t="n">
-        <v>16.13</v>
+        <v>14.27</v>
       </c>
       <c r="Q6" t="n">
-        <v>-112</v>
+        <v>107</v>
       </c>
       <c r="R6" t="n">
-        <v>2406</v>
+        <v>-886</v>
       </c>
       <c r="S6" t="n">
-        <v>-795</v>
+        <v>-408</v>
       </c>
       <c r="T6" t="n">
-        <v>-664</v>
+        <v>-699</v>
       </c>
       <c r="U6" t="n">
-        <v>552</v>
+        <v>806</v>
       </c>
       <c r="V6" t="n">
-        <v>-435</v>
+        <v>-47</v>
       </c>
       <c r="W6" t="n">
         <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>-435</v>
+        <v>-47</v>
       </c>
       <c r="Y6" t="n">
-        <v>3818</v>
+        <v>3086</v>
       </c>
       <c r="Z6" t="n">
-        <v>25.98</v>
+        <v>40.84</v>
       </c>
       <c r="AA6" t="n">
-        <v>4410</v>
+        <v>1978</v>
       </c>
       <c r="AB6" t="n">
-        <v>2289</v>
+        <v>2031</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.35</v>
+        <v>0.39</v>
       </c>
       <c r="AD6" t="n">
-        <v>9.25</v>
+        <v>103.39</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
@@ -1610,476 +1610,571 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45473</v>
+        <v>45565</v>
       </c>
       <c r="B7" t="n">
-        <v>76.7</v>
+        <v>67.14</v>
       </c>
       <c r="C7" t="n">
-        <v>19.41</v>
+        <v>22.44</v>
       </c>
       <c r="D7" t="n">
-        <v>5.15</v>
+        <v>4.46</v>
       </c>
       <c r="E7" t="n">
-        <v>1794</v>
+        <v>2128</v>
       </c>
       <c r="F7" t="n">
-        <v>14.87</v>
+        <v>18.32</v>
       </c>
       <c r="G7" t="n">
-        <v>5.46</v>
+        <v>6.41</v>
       </c>
       <c r="H7" t="n">
-        <v>62436150</v>
+        <v>80572460</v>
       </c>
       <c r="I7" t="n">
-        <v>8444</v>
+        <v>8412</v>
       </c>
       <c r="J7" t="n">
-        <v>383</v>
+        <v>1882</v>
       </c>
       <c r="K7" t="n">
-        <v>8061</v>
+        <v>6530</v>
       </c>
       <c r="L7" t="n">
-        <v>1.3</v>
+        <v>0.93</v>
       </c>
       <c r="M7" t="n">
-        <v>0.71</v>
+        <v>0.52</v>
       </c>
       <c r="N7" t="n">
-        <v>11.4</v>
+        <v>12.4</v>
       </c>
       <c r="O7" t="n">
-        <v>28.54</v>
+        <v>28.86</v>
       </c>
       <c r="P7" t="n">
-        <v>13.55</v>
+        <v>16.13</v>
       </c>
       <c r="Q7" t="n">
-        <v>-613</v>
+        <v>-112</v>
       </c>
       <c r="R7" t="n">
-        <v>1820</v>
+        <v>2406</v>
       </c>
       <c r="S7" t="n">
-        <v>-1469</v>
+        <v>-795</v>
       </c>
       <c r="T7" t="n">
-        <v>-1159</v>
+        <v>-664</v>
       </c>
       <c r="U7" t="n">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="V7" t="n">
-        <v>-264</v>
+        <v>-435</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>-264</v>
+        <v>-435</v>
       </c>
       <c r="Y7" t="n">
-        <v>2051</v>
+        <v>3818</v>
       </c>
       <c r="Z7" t="n">
-        <v>47.94</v>
+        <v>25.98</v>
       </c>
       <c r="AA7" t="n">
-        <v>4212</v>
+        <v>4410</v>
       </c>
       <c r="AB7" t="n">
-        <v>1699</v>
+        <v>2289</v>
       </c>
       <c r="AC7" t="n">
         <v>0.35</v>
       </c>
       <c r="AD7" t="n">
-        <v>13.51</v>
+        <v>9.25</v>
       </c>
       <c r="AE7" t="n">
-        <v>500000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45382</v>
+        <v>45473</v>
       </c>
       <c r="B8" t="n">
-        <v>65.58</v>
+        <v>76.58</v>
       </c>
       <c r="C8" t="n">
-        <v>23.06</v>
+        <v>19.38</v>
       </c>
       <c r="D8" t="n">
-        <v>4.34</v>
+        <v>5.16</v>
       </c>
       <c r="E8" t="n">
-        <v>1507</v>
+        <v>1794</v>
       </c>
       <c r="F8" t="n">
-        <v>14.33</v>
+        <v>14.87</v>
       </c>
       <c r="G8" t="n">
-        <v>5.17</v>
+        <v>5.46</v>
       </c>
       <c r="H8" t="n">
-        <v>57906390</v>
+        <v>62338500</v>
       </c>
       <c r="I8" t="n">
-        <v>8474</v>
+        <v>8444</v>
       </c>
       <c r="J8" t="n">
-        <v>645</v>
+        <v>383</v>
       </c>
       <c r="K8" t="n">
-        <v>7829</v>
+        <v>8061</v>
       </c>
       <c r="L8" t="n">
-        <v>1.56</v>
+        <v>1.3</v>
       </c>
       <c r="M8" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="N8" t="n">
-        <v>13.08</v>
+        <v>11.39</v>
       </c>
       <c r="O8" t="n">
-        <v>22.71</v>
+        <v>28.54</v>
       </c>
       <c r="P8" t="n">
-        <v>8.369999999999999</v>
+        <v>13.55</v>
       </c>
       <c r="Q8" t="n">
-        <v>-723</v>
+        <v>-613</v>
       </c>
       <c r="R8" t="n">
-        <v>830</v>
+        <v>1820</v>
       </c>
       <c r="S8" t="n">
-        <v>84</v>
+        <v>-1469</v>
       </c>
       <c r="T8" t="n">
-        <v>-1461</v>
+        <v>-1159</v>
       </c>
       <c r="U8" t="n">
-        <v>738</v>
+        <v>546</v>
       </c>
       <c r="V8" t="n">
-        <v>-61</v>
+        <v>-264</v>
       </c>
       <c r="W8" t="n">
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>-61</v>
+        <v>-264</v>
       </c>
       <c r="Y8" t="n">
-        <v>2538</v>
+        <v>2051</v>
       </c>
       <c r="Z8" t="n">
-        <v>107.65</v>
+        <v>47.94</v>
       </c>
       <c r="AA8" t="n">
-        <v>4707</v>
+        <v>4212</v>
       </c>
       <c r="AB8" t="n">
-        <v>325</v>
+        <v>1699</v>
       </c>
       <c r="AC8" t="n">
         <v>0.35</v>
       </c>
       <c r="AD8" t="n">
-        <v>12.68</v>
+        <v>13.51</v>
       </c>
       <c r="AE8" t="n">
-        <v>499000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45199</v>
+        <v>45382</v>
       </c>
       <c r="B9" t="n">
-        <v>47.28</v>
+        <v>65.48</v>
       </c>
       <c r="C9" t="n">
-        <v>23.54</v>
+        <v>23.03</v>
       </c>
       <c r="D9" t="n">
-        <v>4.25</v>
+        <v>4.34</v>
       </c>
       <c r="E9" t="n">
-        <v>1598</v>
+        <v>1507</v>
       </c>
       <c r="F9" t="n">
-        <v>11.96</v>
+        <v>14.33</v>
       </c>
       <c r="G9" t="n">
-        <v>2.96</v>
+        <v>5.16</v>
       </c>
       <c r="H9" t="n">
-        <v>34560260</v>
+        <v>57814460</v>
       </c>
       <c r="I9" t="n">
-        <v>7628</v>
+        <v>8474</v>
       </c>
       <c r="J9" t="n">
-        <v>1977</v>
+        <v>645</v>
       </c>
       <c r="K9" t="n">
-        <v>5651</v>
+        <v>7829</v>
       </c>
       <c r="L9" t="n">
-        <v>1.39</v>
+        <v>1.56</v>
       </c>
       <c r="M9" t="n">
-        <v>0.48</v>
+        <v>0.7</v>
       </c>
       <c r="N9" t="n">
-        <v>9.859999999999999</v>
+        <v>13.07</v>
       </c>
       <c r="O9" t="n">
-        <v>12.62</v>
+        <v>22.71</v>
       </c>
       <c r="P9" t="n">
-        <v>5.6</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="Q9" t="n">
-        <v>-993</v>
+        <v>-723</v>
       </c>
       <c r="R9" t="n">
-        <v>2008</v>
+        <v>830</v>
       </c>
       <c r="S9" t="n">
-        <v>637</v>
+        <v>84</v>
       </c>
       <c r="T9" t="n">
-        <v>-1392</v>
+        <v>-1461</v>
       </c>
       <c r="U9" t="n">
-        <v>399</v>
+        <v>738</v>
       </c>
       <c r="V9" t="n">
-        <v>-418</v>
+        <v>-61</v>
       </c>
       <c r="W9" t="n">
         <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>-418</v>
+        <v>-61</v>
       </c>
       <c r="Y9" t="n">
-        <v>4639</v>
+        <v>2538</v>
       </c>
       <c r="Z9" t="n">
-        <v>172.16</v>
+        <v>107.65</v>
       </c>
       <c r="AA9" t="n">
-        <v>2949</v>
+        <v>4707</v>
       </c>
       <c r="AB9" t="n">
-        <v>-600</v>
+        <v>325</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.29</v>
+        <v>0.35</v>
       </c>
       <c r="AD9" t="n">
-        <v>12.59</v>
+        <v>12.68</v>
       </c>
       <c r="AE9" t="n">
-        <v>251000</v>
+        <v>499000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45107</v>
+        <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>34.94</v>
+        <v>47.2</v>
       </c>
       <c r="C10" t="n">
-        <v>46.07</v>
+        <v>23.5</v>
       </c>
       <c r="D10" t="n">
-        <v>2.17</v>
+        <v>4.26</v>
       </c>
       <c r="E10" t="n">
-        <v>1283</v>
+        <v>1598</v>
       </c>
       <c r="F10" t="n">
-        <v>15.3</v>
+        <v>11.96</v>
       </c>
       <c r="G10" t="n">
-        <v>2.59</v>
+        <v>2.96</v>
       </c>
       <c r="H10" t="n">
-        <v>29108160</v>
+        <v>34505520</v>
       </c>
       <c r="I10" t="n">
-        <v>6266</v>
+        <v>7628</v>
       </c>
       <c r="J10" t="n">
-        <v>325</v>
+        <v>1977</v>
       </c>
       <c r="K10" t="n">
-        <v>5941</v>
+        <v>5651</v>
       </c>
       <c r="L10" t="n">
-        <v>1.77</v>
+        <v>1.39</v>
       </c>
       <c r="M10" t="n">
-        <v>0.53</v>
+        <v>0.48</v>
       </c>
       <c r="N10" t="n">
-        <v>10.44</v>
+        <v>9.84</v>
       </c>
       <c r="O10" t="n">
+        <v>12.62</v>
+      </c>
+      <c r="P10" t="n">
         <v>5.6</v>
       </c>
-      <c r="P10" t="n">
-        <v>5.19</v>
-      </c>
       <c r="Q10" t="n">
-        <v>-192</v>
+        <v>-993</v>
       </c>
       <c r="R10" t="n">
-        <v>-48</v>
+        <v>2008</v>
       </c>
       <c r="S10" t="n">
-        <v>229</v>
+        <v>637</v>
       </c>
       <c r="T10" t="n">
-        <v>-868</v>
+        <v>-1392</v>
       </c>
       <c r="U10" t="n">
-        <v>676</v>
+        <v>399</v>
       </c>
       <c r="V10" t="n">
-        <v>-411</v>
+        <v>-418</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>-411</v>
+        <v>-418</v>
       </c>
       <c r="Y10" t="n">
-        <v>2350</v>
+        <v>4639</v>
       </c>
       <c r="Z10" t="n">
-        <v>85.15000000000001</v>
+        <v>172.16</v>
       </c>
       <c r="AA10" t="n">
-        <v>868</v>
+        <v>2949</v>
       </c>
       <c r="AB10" t="n">
-        <v>-115</v>
+        <v>-600</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.28</v>
+        <v>0.29</v>
       </c>
       <c r="AD10" t="n">
-        <v>11.04</v>
+        <v>12.59</v>
       </c>
       <c r="AE10" t="n">
-        <v>268000</v>
+        <v>251000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45016</v>
+        <v>45107</v>
       </c>
       <c r="B11" t="n">
-        <v>262.26</v>
+        <v>34.89</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.39</v>
+        <v>2.17</v>
       </c>
       <c r="E11" t="n">
-        <v>636</v>
+        <v>1283</v>
       </c>
       <c r="F11" t="n">
-        <v>1.27</v>
+        <v>15.3</v>
       </c>
       <c r="G11" t="n">
-        <v>2.35</v>
+        <v>2.58</v>
       </c>
       <c r="H11" t="n">
-        <v>25177280</v>
+        <v>29062800</v>
       </c>
       <c r="I11" t="n">
-        <v>5924</v>
+        <v>6266</v>
       </c>
       <c r="J11" t="n">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="K11" t="n">
-        <v>5588</v>
+        <v>5941</v>
       </c>
       <c r="L11" t="n">
-        <v>1.8</v>
+        <v>1.77</v>
       </c>
       <c r="M11" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="N11" t="n">
-        <v>9.890000000000001</v>
+        <v>10.42</v>
       </c>
       <c r="O11" t="n">
-        <v>-0.9</v>
+        <v>5.6</v>
       </c>
       <c r="P11" t="n">
-        <v>6.43</v>
+        <v>5.19</v>
       </c>
       <c r="Q11" t="n">
-        <v>-934</v>
+        <v>-192</v>
       </c>
       <c r="R11" t="n">
-        <v>219</v>
+        <v>-48</v>
       </c>
       <c r="S11" t="n">
-        <v>523</v>
+        <v>229</v>
       </c>
       <c r="T11" t="n">
-        <v>-1594</v>
+        <v>-868</v>
       </c>
       <c r="U11" t="n">
-        <v>660</v>
+        <v>676</v>
       </c>
       <c r="V11" t="n">
-        <v>-665</v>
+        <v>-411</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>-665</v>
+        <v>-411</v>
       </c>
       <c r="Y11" t="n">
-        <v>2161</v>
+        <v>2350</v>
       </c>
       <c r="Z11" t="n">
-        <v>102.34</v>
+        <v>85.15000000000001</v>
       </c>
       <c r="AA11" t="n">
-        <v>-1883</v>
+        <v>868</v>
       </c>
       <c r="AB11" t="n">
-        <v>-782</v>
+        <v>-115</v>
       </c>
       <c r="AC11" t="n">
         <v>0.28</v>
       </c>
       <c r="AD11" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>268000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>45016</v>
+      </c>
+      <c r="B12" t="n">
+        <v>261.85</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="E12" t="n">
+        <v>636</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="H12" t="n">
+        <v>25137920</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5924</v>
+      </c>
+      <c r="J12" t="n">
+        <v>336</v>
+      </c>
+      <c r="K12" t="n">
+        <v>5588</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="N12" t="n">
+        <v>9.869999999999999</v>
+      </c>
+      <c r="O12" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="P12" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>-934</v>
+      </c>
+      <c r="R12" t="n">
+        <v>219</v>
+      </c>
+      <c r="S12" t="n">
+        <v>523</v>
+      </c>
+      <c r="T12" t="n">
+        <v>-1594</v>
+      </c>
+      <c r="U12" t="n">
+        <v>660</v>
+      </c>
+      <c r="V12" t="n">
+        <v>-665</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" t="n">
+        <v>-665</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>2161</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>102.34</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>-1883</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>-782</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="AD12" t="n">
         <v>96.88</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AE12" t="n">
         <v>231000</v>
       </c>
     </row>

</xml_diff>